<commit_message>
fixing all about " Ability to be filled " parameter, README.md updating
</commit_message>
<xml_diff>
--- a/Data of timepoint 2.xlsx
+++ b/Data of timepoint 2.xlsx
@@ -710,7 +710,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -719,8 +719,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1121,7 +1120,7 @@
         <v>5</v>
       </c>
       <c r="H2" s="4">
-        <v>0.7476</v>
+        <v>74.76</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1150,7 +1149,7 @@
         <v>12</v>
       </c>
       <c r="H3" s="4">
-        <v>0.607</v>
+        <v>60.7</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1178,8 +1177,8 @@
       <c r="G4">
         <v>6</v>
       </c>
-      <c r="H4" s="5">
-        <v>0.6</v>
+      <c r="H4" s="4">
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1207,8 +1206,8 @@
       <c r="G5">
         <v>2</v>
       </c>
-      <c r="H5" s="5">
-        <v>0.5</v>
+      <c r="H5" s="4">
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1237,7 +1236,7 @@
         <v>6</v>
       </c>
       <c r="H6" s="4">
-        <v>0.5133</v>
+        <v>51.33</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1266,7 +1265,7 @@
         <v>2</v>
       </c>
       <c r="H7" s="4">
-        <v>0.5375</v>
+        <v>53.75</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1295,7 +1294,7 @@
         <v>2</v>
       </c>
       <c r="H8" s="4">
-        <v>0.2082</v>
+        <v>20.82</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1323,7 +1322,7 @@
         <v>2</v>
       </c>
       <c r="H9" s="4">
-        <v>0.226</v>
+        <v>22.6</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1352,7 +1351,7 @@
         <v>3</v>
       </c>
       <c r="H10" s="4">
-        <v>0.4175</v>
+        <v>41.75</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1381,7 +1380,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="4">
-        <v>0.4417</v>
+        <v>44.17</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1410,7 +1409,7 @@
         <v>2</v>
       </c>
       <c r="H12" s="4">
-        <v>0.378</v>
+        <v>37.8</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1438,8 +1437,8 @@
       <c r="G13">
         <v>3</v>
       </c>
-      <c r="H13" s="5">
-        <v>0.4</v>
+      <c r="H13" s="4">
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -1467,8 +1466,8 @@
       <c r="G14">
         <v>3</v>
       </c>
-      <c r="H14" s="5">
-        <v>0.475</v>
+      <c r="H14" s="4">
+        <v>47.5</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1497,7 +1496,7 @@
         <v>3</v>
       </c>
       <c r="H15" s="4">
-        <v>0.566</v>
+        <v>56.6</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1526,7 +1525,7 @@
         <v>4</v>
       </c>
       <c r="H16" s="4">
-        <v>0.225</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1555,7 +1554,7 @@
         <v>3</v>
       </c>
       <c r="H17" s="4">
-        <v>0.3225</v>
+        <v>32.25</v>
       </c>
     </row>
     <row r="18" ht="13.5" customHeight="1"/>

</xml_diff>